<commit_message>
chore: merge in batch changes
</commit_message>
<xml_diff>
--- a/tests/data/gen_spaces_test.xlsx
+++ b/tests/data/gen_spaces_test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3ac2bf50d090347/Documents/Python/Neontribe/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3ac2bf50d090347/Documents/Python/Neontribe/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="6" documentId="8_{CA5381B8-E57E-40F0-8282-1E0882E13D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A35A3585-4800-4BE8-9411-DABA4411C79F}"/>
@@ -579,10 +579,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>